<commit_message>
Fix Our Notes footer duplication on rebuild; verify note round-trip
</commit_message>
<xml_diff>
--- a/Pillar4_Stock_Notes.xlsx
+++ b/Pillar4_Stock_Notes.xlsx
@@ -19,7 +19,7 @@
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Comment Log'!$A$1:$D$1452</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Dashboard Notes'!$A$1:$C$38</definedName>
     <definedName function="false" hidden="true" localSheetId="5" name="_xlnm._FilterDatabase" vbProcedure="false">'Follow-ups'!$A$1:$D$20</definedName>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Our Notes'!$A$1:$F$3</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'Our Notes'!$A$1:$F$2</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Stock Index'!$A$1:$M$127</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6990" uniqueCount="1220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6989" uniqueCount="1220">
   <si>
     <t xml:space="preserve">PILLAR 4 - US STOCK NOTES</t>
   </si>
@@ -3793,7 +3793,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3810,6 +3810,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
         <bgColor rgb="FF333333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -3862,7 +3868,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3911,6 +3917,10 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3924,7 +3934,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="5">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3952,6 +3962,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF006100"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFF00"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -29945,7 +29963,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="12"/>
@@ -29976,7 +29994,7 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="12" t="s">
         <v>4</v>
       </c>
       <c r="B2" s="10" t="s">
@@ -29995,23 +30013,13 @@
         <v>1176</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="s">
         <v>1177</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>1177</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F3"/>
+  <autoFilter ref="A1:F2"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>